<commit_message>
Second Commit ----- SUREFIRE PLUGIN
</commit_message>
<xml_diff>
--- a/testData/demoWebShopAssignment.xlsx
+++ b/testData/demoWebShopAssignment.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
   <si>
     <t>Country</t>
   </si>
@@ -93,6 +93,12 @@
   </si>
   <si>
     <t>2239661</t>
+  </si>
+  <si>
+    <t>2239663</t>
+  </si>
+  <si>
+    <t>2239668</t>
   </si>
 </sst>
 </file>
@@ -524,7 +530,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes in POM.xml Snapshot 0.0.1
</commit_message>
<xml_diff>
--- a/testData/demoWebShopAssignment.xlsx
+++ b/testData/demoWebShopAssignment.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
   <si>
     <t>Country</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>2239668</t>
+  </si>
+  <si>
+    <t>2239674</t>
   </si>
 </sst>
 </file>
@@ -530,7 +533,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Executed mvn clean install in the cmd
</commit_message>
<xml_diff>
--- a/testData/demoWebShopAssignment.xlsx
+++ b/testData/demoWebShopAssignment.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
   <si>
     <t>Country</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t>2239674</t>
+  </si>
+  <si>
+    <t>2239679</t>
   </si>
 </sst>
 </file>
@@ -533,7 +536,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Commit --- latest Commit as on 09-03-26 ----- Added LIstenerClass and ThreadLocal Class
</commit_message>
<xml_diff>
--- a/testData/demoWebShopAssignment.xlsx
+++ b/testData/demoWebShopAssignment.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>Country</t>
   </si>
@@ -105,6 +105,18 @@
   </si>
   <si>
     <t>2239679</t>
+  </si>
+  <si>
+    <t>2240337</t>
+  </si>
+  <si>
+    <t>2240340</t>
+  </si>
+  <si>
+    <t>2240348</t>
+  </si>
+  <si>
+    <t>2240356</t>
   </si>
 </sst>
 </file>
@@ -536,7 +548,7 @@
   <sheetData>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>